<commit_message>
completed ICAI, and IBBI Discussion paper, also added in my windows codes copy folder,All sprints arenow completed except MCA
</commit_message>
<xml_diff>
--- a/data/Links.xlsx
+++ b/data/Links.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="SEBI"/>
     <sheet r:id="rId2" sheetId="2" name="Listed Companies"/>
-    <sheet r:id="rId3" sheetId="3" name="IFSCA"/>
+    <sheet r:id="rId3" sheetId="3" name="ICAI"/>
     <sheet r:id="rId4" sheetId="4" name="RBI"/>
     <sheet r:id="rId5" sheetId="5" name="IBBI"/>
   </sheets>
@@ -18,18 +18,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
   <si>
     <t>IBBI - Litigation</t>
   </si>
   <si>
-    <t/>
+    <t>Discussion Paper</t>
+  </si>
+  <si>
+    <t>https://ibbi.gov.in//en/public-comments/comments-on</t>
   </si>
   <si>
     <t>RBI</t>
   </si>
   <si>
-    <t>IFSCA - Gift</t>
+    <t>ICAI</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>Listed Companies</t>
@@ -37,19 +43,13 @@
   <si>
     <t>SEBI</t>
   </si>
-  <si>
-    <t>Informal Guidance</t>
-  </si>
-  <si>
-    <t>https://www.sebi.gov.in/sebiweb/home/HomeAction.do?doListing=yes&amp;sid=2&amp;ssid=10&amp;smid=0</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -68,6 +68,12 @@
       <sz val="11"/>
       <color rgb="FF1155cc"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -141,44 +147,44 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="4" applyFill="1" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -485,38 +491,38 @@
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="75.14785714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="75.14785714285713" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="5" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -544,12 +550,8 @@
       <c r="Z1" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
-      <c r="A2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>7</v>
-      </c>
+      <c r="A2" s="1"/>
+      <c r="B2" s="11"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -576,12 +578,8 @@
       <c r="Z2" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
-      <c r="A3" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A3" s="1"/>
+      <c r="B3" s="3"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -608,12 +606,8 @@
       <c r="Z3" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
-      <c r="A4" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="3"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -640,12 +634,8 @@
       <c r="Z4" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
-      <c r="A5" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="3"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -672,12 +662,8 @@
       <c r="Z5" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
-      <c r="A6" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A6" s="1"/>
+      <c r="B6" s="3"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -704,12 +690,8 @@
       <c r="Z6" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
-      <c r="A7" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" s="15" t="s">
-        <v>1</v>
-      </c>
+      <c r="A7" s="1"/>
+      <c r="B7" s="11"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -28552,33 +28534,33 @@
   <dimension ref="A1:U1001"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="11" width="61.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="12" width="61.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="5" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -28601,12 +28583,8 @@
       <c r="U1" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A2" s="1"/>
+      <c r="B2" s="3"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -28628,12 +28606,8 @@
       <c r="U2" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
-      <c r="A3" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A3" s="1"/>
+      <c r="B3" s="3"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -28655,8 +28629,8 @@
       <c r="U3" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
-      <c r="A4" s="12"/>
-      <c r="B4" s="13"/>
+      <c r="A4" s="13"/>
+      <c r="B4" s="14"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -51560,53 +51534,53 @@
       <c r="R999" s="1"/>
       <c r="S999" s="1"/>
       <c r="T999" s="1"/>
-      <c r="U999" s="12"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="1000" customHeight="1" ht="18" customFormat="1" s="14">
-      <c r="A1000" s="13"/>
+      <c r="U999" s="13"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="1000" customHeight="1" ht="18" customFormat="1" s="15">
+      <c r="A1000" s="14"/>
       <c r="B1000" s="2"/>
-      <c r="C1000" s="13"/>
-      <c r="D1000" s="13"/>
-      <c r="E1000" s="13"/>
-      <c r="F1000" s="13"/>
-      <c r="G1000" s="13"/>
-      <c r="H1000" s="13"/>
-      <c r="I1000" s="13"/>
-      <c r="J1000" s="13"/>
-      <c r="K1000" s="13"/>
-      <c r="L1000" s="13"/>
-      <c r="M1000" s="13"/>
-      <c r="N1000" s="13"/>
-      <c r="O1000" s="13"/>
-      <c r="P1000" s="13"/>
-      <c r="Q1000" s="13"/>
-      <c r="R1000" s="13"/>
-      <c r="S1000" s="13"/>
-      <c r="T1000" s="13"/>
-      <c r="U1000" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="1001" customHeight="1" ht="18" customFormat="1" s="14">
-      <c r="A1001" s="13"/>
+      <c r="C1000" s="14"/>
+      <c r="D1000" s="14"/>
+      <c r="E1000" s="14"/>
+      <c r="F1000" s="14"/>
+      <c r="G1000" s="14"/>
+      <c r="H1000" s="14"/>
+      <c r="I1000" s="14"/>
+      <c r="J1000" s="14"/>
+      <c r="K1000" s="14"/>
+      <c r="L1000" s="14"/>
+      <c r="M1000" s="14"/>
+      <c r="N1000" s="14"/>
+      <c r="O1000" s="14"/>
+      <c r="P1000" s="14"/>
+      <c r="Q1000" s="14"/>
+      <c r="R1000" s="14"/>
+      <c r="S1000" s="14"/>
+      <c r="T1000" s="14"/>
+      <c r="U1000" s="14"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="1001" customHeight="1" ht="18" customFormat="1" s="15">
+      <c r="A1001" s="14"/>
       <c r="B1001" s="2"/>
-      <c r="C1001" s="13"/>
-      <c r="D1001" s="13"/>
-      <c r="E1001" s="13"/>
-      <c r="F1001" s="13"/>
-      <c r="G1001" s="13"/>
-      <c r="H1001" s="13"/>
-      <c r="I1001" s="13"/>
-      <c r="J1001" s="13"/>
-      <c r="K1001" s="13"/>
-      <c r="L1001" s="13"/>
-      <c r="M1001" s="13"/>
-      <c r="N1001" s="13"/>
-      <c r="O1001" s="13"/>
-      <c r="P1001" s="13"/>
-      <c r="Q1001" s="13"/>
-      <c r="R1001" s="13"/>
-      <c r="S1001" s="13"/>
-      <c r="T1001" s="13"/>
-      <c r="U1001" s="13"/>
+      <c r="C1001" s="14"/>
+      <c r="D1001" s="14"/>
+      <c r="E1001" s="14"/>
+      <c r="F1001" s="14"/>
+      <c r="G1001" s="14"/>
+      <c r="H1001" s="14"/>
+      <c r="I1001" s="14"/>
+      <c r="J1001" s="14"/>
+      <c r="K1001" s="14"/>
+      <c r="L1001" s="14"/>
+      <c r="M1001" s="14"/>
+      <c r="N1001" s="14"/>
+      <c r="O1001" s="14"/>
+      <c r="P1001" s="14"/>
+      <c r="Q1001" s="14"/>
+      <c r="R1001" s="14"/>
+      <c r="S1001" s="14"/>
+      <c r="T1001" s="14"/>
+      <c r="U1001" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -51621,75 +51595,51 @@
   <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="11" width="40.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="12" width="40.57642857142857" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
+      <c r="A2" s="8" t="s">
+        <v>5</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>1</v>
+      <c r="B2" s="9" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
-      <c r="A3" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
-      <c r="A4" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
-      <c r="A5" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
-      <c r="A6" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
-      <c r="A7" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18">
-      <c r="A8" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="1"/>
+      <c r="B3" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="1"/>
+      <c r="B4" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="1"/>
+      <c r="B5" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="10"/>
+      <c r="B6" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="10"/>
+      <c r="B7" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="10"/>
+      <c r="B8" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1"/>
-      <c r="B9" s="10"/>
+      <c r="B9" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -51704,63 +51654,39 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="48.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="48.86214285714286" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
-      <c r="A2" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A2" s="6"/>
+      <c r="B2" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
-      <c r="A3" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A3" s="7"/>
+      <c r="B3" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
-      <c r="A4" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A4" s="6"/>
+      <c r="B4" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
-      <c r="A5" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A5" s="7"/>
+      <c r="B5" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
-      <c r="A6" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A6" s="6"/>
+      <c r="B6" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
-      <c r="A7" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A7" s="6"/>
+      <c r="B7" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18">
       <c r="A8" s="1"/>
@@ -51779,8 +51705,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="41.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="41.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
@@ -51790,52 +51716,32 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>1</v>
+      <c r="B2" s="3" t="s">
+        <v>2</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
-      <c r="A3" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A3" s="1"/>
+      <c r="B3" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
-      <c r="A4" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
-      <c r="A5" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>1</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
-      <c r="A6" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>1</v>
-      </c>
+      <c r="A6" s="1"/>
+      <c r="B6" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
-      <c r="A7" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A7" s="1"/>
+      <c r="B7" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
changed public consulataion approach
</commit_message>
<xml_diff>
--- a/data/Links.xlsx
+++ b/data/Links.xlsx
@@ -4,12 +4,12 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="SEBI"/>
     <sheet r:id="rId2" sheetId="2" name="Listed Companies"/>
-    <sheet r:id="rId3" sheetId="3" name="ICAI"/>
+    <sheet r:id="rId3" sheetId="3" name="IFSCA"/>
     <sheet r:id="rId4" sheetId="4" name="RBI"/>
     <sheet r:id="rId5" sheetId="5" name="IBBI"/>
   </sheets>
@@ -18,33 +18,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="8">
   <si>
     <t>IBBI - Litigation</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>RBI</t>
   </si>
   <si>
-    <t>ICAI</t>
+    <t>IFSCA</t>
+  </si>
+  <si>
+    <t>Public Consultation</t>
+  </si>
+  <si>
+    <t>https://ifsca.gov.in/ReportPublication/index/sKCVtbX6J9o=</t>
   </si>
   <si>
     <t>Listed Companies</t>
   </si>
   <si>
-    <t>Circular-BSE</t>
-  </si>
-  <si>
-    <t>https://www.bseindia.com/corporates/CirularToListedComp.html</t>
-  </si>
-  <si>
-    <t>Circular-NSE</t>
-  </si>
-  <si>
-    <t>https://www.nseindia.com/companies-listing/circular-for-listed-companies-equity-market</t>
+    <t/>
   </si>
   <si>
     <t>SEBI</t>
@@ -55,7 +49,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -74,12 +68,6 @@
       <sz val="11"/>
       <color rgb="FF1155cc"/>
       <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
@@ -159,12 +147,6 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -189,10 +171,16 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -503,38 +491,38 @@
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="75.14785714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="75.14785714285713" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="5" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -561,9 +549,9 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1"/>
-      <c r="B2" s="11"/>
+      <c r="B2" s="9"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -589,9 +577,9 @@
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1"/>
-      <c r="B3" s="5"/>
+      <c r="B3" s="3"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -617,9 +605,9 @@
       <c r="Y3" s="1"/>
       <c r="Z3" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1"/>
-      <c r="B4" s="5"/>
+      <c r="B4" s="3"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -645,9 +633,9 @@
       <c r="Y4" s="1"/>
       <c r="Z4" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1"/>
-      <c r="B5" s="5"/>
+      <c r="B5" s="3"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -673,9 +661,9 @@
       <c r="Y5" s="1"/>
       <c r="Z5" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1"/>
-      <c r="B6" s="5"/>
+      <c r="B6" s="3"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -701,9 +689,9 @@
       <c r="Y6" s="1"/>
       <c r="Z6" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1"/>
-      <c r="B7" s="11"/>
+      <c r="B7" s="9"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -729,7 +717,7 @@
       <c r="Y7" s="1"/>
       <c r="Z7" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -757,7 +745,7 @@
       <c r="Y8" s="1"/>
       <c r="Z8" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -785,7 +773,7 @@
       <c r="Y9" s="1"/>
       <c r="Z9" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -813,7 +801,7 @@
       <c r="Y10" s="1"/>
       <c r="Z10" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -841,7 +829,7 @@
       <c r="Y11" s="1"/>
       <c r="Z11" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -869,7 +857,7 @@
       <c r="Y12" s="1"/>
       <c r="Z12" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -897,7 +885,7 @@
       <c r="Y13" s="1"/>
       <c r="Z13" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -925,7 +913,7 @@
       <c r="Y14" s="1"/>
       <c r="Z14" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -28546,33 +28534,33 @@
   <dimension ref="A1:U1001"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="12" width="61.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="10" width="61.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="5" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -28595,10 +28583,10 @@
       <c r="U1" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
+      <c r="A2" s="11" t="s">
+        <v>6</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="12" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="1"/>
@@ -28622,11 +28610,11 @@
       <c r="U2" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
-      <c r="A3" s="1" t="s">
-        <v>7</v>
+      <c r="A3" s="11" t="s">
+        <v>6</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>8</v>
+      <c r="B3" s="12" t="s">
+        <v>6</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -51615,47 +51603,51 @@
   <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="12" width="40.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="10" width="40.57642857142857" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+      <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="1"/>
-      <c r="B2" s="5"/>
+      <c r="B2" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1"/>
-      <c r="B3" s="5"/>
+      <c r="B3" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1"/>
-      <c r="B4" s="5"/>
+      <c r="B4" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1"/>
-      <c r="B5" s="5"/>
+      <c r="B5" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="10"/>
-      <c r="B6" s="5"/>
+      <c r="A6" s="8"/>
+      <c r="B6" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="10"/>
-      <c r="B7" s="5"/>
+      <c r="A7" s="8"/>
+      <c r="B7" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="10"/>
-      <c r="B8" s="5"/>
+      <c r="A8" s="8"/>
+      <c r="B8" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1"/>
-      <c r="B9" s="11"/>
+      <c r="B9" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -51670,39 +51662,39 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="48.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="48.86214285714286" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
-      <c r="A2" s="8"/>
-      <c r="B2" s="5"/>
+      <c r="A2" s="6"/>
+      <c r="B2" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
-      <c r="A3" s="9"/>
-      <c r="B3" s="5"/>
+      <c r="A3" s="7"/>
+      <c r="B3" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
-      <c r="A4" s="8"/>
-      <c r="B4" s="5"/>
+      <c r="A4" s="6"/>
+      <c r="B4" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
-      <c r="A5" s="9"/>
-      <c r="B5" s="5"/>
+      <c r="A5" s="7"/>
+      <c r="B5" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
-      <c r="A6" s="8"/>
-      <c r="B6" s="5"/>
+      <c r="A6" s="6"/>
+      <c r="B6" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
-      <c r="A7" s="8"/>
-      <c r="B7" s="5"/>
+      <c r="A7" s="6"/>
+      <c r="B7" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18">
       <c r="A8" s="1"/>
@@ -51721,8 +51713,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="41.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="41.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
@@ -51732,32 +51724,28 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A2" s="1"/>
+      <c r="B2" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
       <c r="A3" s="1"/>
-      <c r="B3" s="5"/>
+      <c r="B3" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
       <c r="A4" s="1"/>
-      <c r="B4" s="5"/>
+      <c r="B4" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
       <c r="A5" s="1"/>
-      <c r="B5" s="6"/>
+      <c r="B5" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
       <c r="A6" s="1"/>
-      <c r="B6" s="6"/>
+      <c r="B6" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
       <c r="A7" s="1"/>
-      <c r="B7" s="5"/>
+      <c r="B7" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added Companies Act(MCA) to Searching agent(3 subdomains),added the old parsing agent code without mca sql_db or mca_ui
</commit_message>
<xml_diff>
--- a/data/Links.xlsx
+++ b/data/Links.xlsx
@@ -9,6 +9,7 @@
     <sheet state="visible" name="RBI" sheetId="4" r:id="rId8"/>
     <sheet state="visible" name="ICAI" sheetId="5" r:id="rId9"/>
     <sheet state="visible" name="IBBI" sheetId="6" r:id="rId10"/>
+    <sheet state="visible" name="Companies Act" sheetId="7" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -16,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="52">
   <si>
     <t>SEBI</t>
   </si>
@@ -161,6 +162,18 @@
   <si>
     <t>https://ibbi.gov.in//en/legal-framework/guidelines</t>
   </si>
+  <si>
+    <t>Companies Act</t>
+  </si>
+  <si>
+    <t>https://www.mca.gov.in/content/mca/global/en/acts-rules/ebooks/notifications.html</t>
+  </si>
+  <si>
+    <t>https://www.mca.gov.in/content/mca/global/en/acts-rules/ebooks/circulars.html</t>
+  </si>
+  <si>
+    <t>https://www.mca.gov.in/content/mca/global/en/notifications-tender/news-updates/press-release.html</t>
+  </si>
 </sst>
 </file>
 
@@ -207,7 +220,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -220,6 +233,12 @@
         <bgColor rgb="FFD9EAD3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC9DAF8"/>
+        <bgColor rgb="FFC9DAF8"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -227,7 +246,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -273,6 +292,12 @@
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -302,6 +327,10 @@
 </file>
 
 <file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -51821,4 +51850,55 @@
   </hyperlinks>
   <drawing r:id="rId7"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="15.13"/>
+    <col customWidth="1" min="2" max="2" width="46.75"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15"/>
+      <c r="B1" s="16" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="B2"/>
+    <hyperlink r:id="rId2" ref="B3"/>
+    <hyperlink r:id="rId3" ref="B4"/>
+  </hyperlinks>
+  <drawing r:id="rId4"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
every time sewarching agents runs, it first deletes week range json and searching agent output excel as these are previous weeks results, so that if searching agents fails, the parsing agnets input will be empty
</commit_message>
<xml_diff>
--- a/data/Links.xlsx
+++ b/data/Links.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="SEBI"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="52">
   <si>
     <t>Companies Act</t>
   </si>
@@ -142,16 +142,13 @@
     <t>Listed Companies</t>
   </si>
   <si>
-    <t>Circular-BSE</t>
-  </si>
-  <si>
-    <t>https://www.bseindia.com/corporates/CirularToListedComp.html</t>
-  </si>
-  <si>
     <t>Circular-NSE</t>
   </si>
   <si>
     <t>https://www.nseindia.com/companies-listing/circular-for-listed-companies-equity-market</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>SEBI</t>
@@ -186,7 +183,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -205,6 +202,12 @@
       <sz val="11"/>
       <color rgb="FF1155cc"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -260,7 +263,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -275,10 +278,10 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -289,14 +292,23 @@
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -634,7 +646,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
@@ -666,7 +678,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
@@ -698,7 +710,7 @@
         <v>5</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -727,10 +739,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
       <c r="A4" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -762,7 +774,7 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
@@ -794,7 +806,7 @@
         <v>24</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
@@ -823,10 +835,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
       <c r="A7" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -28670,30 +28682,30 @@
   <dimension ref="A1:U1001"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="15" width="23.290714285714284" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="6" width="61.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
         <v>39</v>
@@ -28718,7 +28730,7 @@
       <c r="T1" s="7"/>
       <c r="U1" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="3" t="s">
         <v>40</v>
       </c>
@@ -28745,12 +28757,12 @@
       <c r="T2" s="7"/>
       <c r="U2" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
-      <c r="A3" s="3" t="s">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
+      <c r="A3" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>43</v>
+      <c r="B3" s="11" t="s">
+        <v>42</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -28772,9 +28784,9 @@
       <c r="T3" s="7"/>
       <c r="U3" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
-      <c r="A4" s="10"/>
-      <c r="B4" s="11"/>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="12"/>
+      <c r="B4" s="13"/>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
@@ -28795,7 +28807,7 @@
       <c r="T4" s="7"/>
       <c r="U4" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="7"/>
       <c r="B5" s="8"/>
       <c r="C5" s="7"/>
@@ -28818,7 +28830,7 @@
       <c r="T5" s="7"/>
       <c r="U5" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="7"/>
       <c r="B6" s="8"/>
       <c r="C6" s="7"/>
@@ -28841,7 +28853,7 @@
       <c r="T6" s="7"/>
       <c r="U6" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="7"/>
       <c r="B7" s="8"/>
       <c r="C7" s="7"/>
@@ -28864,7 +28876,7 @@
       <c r="T7" s="7"/>
       <c r="U7" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="7"/>
       <c r="B8" s="8"/>
       <c r="C8" s="7"/>
@@ -28887,7 +28899,7 @@
       <c r="T8" s="7"/>
       <c r="U8" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="7"/>
       <c r="B9" s="8"/>
       <c r="C9" s="7"/>
@@ -28910,7 +28922,7 @@
       <c r="T9" s="7"/>
       <c r="U9" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="7"/>
       <c r="B10" s="8"/>
       <c r="C10" s="7"/>
@@ -28933,7 +28945,7 @@
       <c r="T10" s="7"/>
       <c r="U10" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="7"/>
       <c r="B11" s="8"/>
       <c r="C11" s="7"/>
@@ -28956,7 +28968,7 @@
       <c r="T11" s="7"/>
       <c r="U11" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="7"/>
       <c r="B12" s="8"/>
       <c r="C12" s="7"/>
@@ -28979,7 +28991,7 @@
       <c r="T12" s="7"/>
       <c r="U12" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="7"/>
       <c r="B13" s="8"/>
       <c r="C13" s="7"/>
@@ -29002,7 +29014,7 @@
       <c r="T13" s="7"/>
       <c r="U13" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="7"/>
       <c r="B14" s="8"/>
       <c r="C14" s="7"/>
@@ -29025,7 +29037,7 @@
       <c r="T14" s="7"/>
       <c r="U14" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="7"/>
       <c r="B15" s="8"/>
       <c r="C15" s="7"/>
@@ -29048,7 +29060,7 @@
       <c r="T15" s="7"/>
       <c r="U15" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="7"/>
       <c r="B16" s="8"/>
       <c r="C16" s="7"/>
@@ -29071,7 +29083,7 @@
       <c r="T16" s="7"/>
       <c r="U16" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="7"/>
       <c r="B17" s="8"/>
       <c r="C17" s="7"/>
@@ -29094,7 +29106,7 @@
       <c r="T17" s="7"/>
       <c r="U17" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="7"/>
       <c r="B18" s="8"/>
       <c r="C18" s="7"/>
@@ -51678,53 +51690,53 @@
       <c r="R999" s="7"/>
       <c r="S999" s="7"/>
       <c r="T999" s="7"/>
-      <c r="U999" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="1000" customHeight="1" ht="17.25" customFormat="1" s="12">
-      <c r="A1000" s="11"/>
+      <c r="U999" s="12"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="1000" customHeight="1" ht="17.25" customFormat="1" s="14">
+      <c r="A1000" s="13"/>
       <c r="B1000" s="8"/>
-      <c r="C1000" s="11"/>
-      <c r="D1000" s="11"/>
-      <c r="E1000" s="11"/>
-      <c r="F1000" s="11"/>
-      <c r="G1000" s="11"/>
-      <c r="H1000" s="11"/>
-      <c r="I1000" s="11"/>
-      <c r="J1000" s="11"/>
-      <c r="K1000" s="11"/>
-      <c r="L1000" s="11"/>
-      <c r="M1000" s="11"/>
-      <c r="N1000" s="11"/>
-      <c r="O1000" s="11"/>
-      <c r="P1000" s="11"/>
-      <c r="Q1000" s="11"/>
-      <c r="R1000" s="11"/>
-      <c r="S1000" s="11"/>
-      <c r="T1000" s="11"/>
-      <c r="U1000" s="11"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="1001" customHeight="1" ht="17.25" customFormat="1" s="12">
-      <c r="A1001" s="11"/>
+      <c r="C1000" s="13"/>
+      <c r="D1000" s="13"/>
+      <c r="E1000" s="13"/>
+      <c r="F1000" s="13"/>
+      <c r="G1000" s="13"/>
+      <c r="H1000" s="13"/>
+      <c r="I1000" s="13"/>
+      <c r="J1000" s="13"/>
+      <c r="K1000" s="13"/>
+      <c r="L1000" s="13"/>
+      <c r="M1000" s="13"/>
+      <c r="N1000" s="13"/>
+      <c r="O1000" s="13"/>
+      <c r="P1000" s="13"/>
+      <c r="Q1000" s="13"/>
+      <c r="R1000" s="13"/>
+      <c r="S1000" s="13"/>
+      <c r="T1000" s="13"/>
+      <c r="U1000" s="13"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="1001" customHeight="1" ht="17.25" customFormat="1" s="14">
+      <c r="A1001" s="13"/>
       <c r="B1001" s="8"/>
-      <c r="C1001" s="11"/>
-      <c r="D1001" s="11"/>
-      <c r="E1001" s="11"/>
-      <c r="F1001" s="11"/>
-      <c r="G1001" s="11"/>
-      <c r="H1001" s="11"/>
-      <c r="I1001" s="11"/>
-      <c r="J1001" s="11"/>
-      <c r="K1001" s="11"/>
-      <c r="L1001" s="11"/>
-      <c r="M1001" s="11"/>
-      <c r="N1001" s="11"/>
-      <c r="O1001" s="11"/>
-      <c r="P1001" s="11"/>
-      <c r="Q1001" s="11"/>
-      <c r="R1001" s="11"/>
-      <c r="S1001" s="11"/>
-      <c r="T1001" s="11"/>
-      <c r="U1001" s="11"/>
+      <c r="C1001" s="13"/>
+      <c r="D1001" s="13"/>
+      <c r="E1001" s="13"/>
+      <c r="F1001" s="13"/>
+      <c r="G1001" s="13"/>
+      <c r="H1001" s="13"/>
+      <c r="I1001" s="13"/>
+      <c r="J1001" s="13"/>
+      <c r="K1001" s="13"/>
+      <c r="L1001" s="13"/>
+      <c r="M1001" s="13"/>
+      <c r="N1001" s="13"/>
+      <c r="O1001" s="13"/>
+      <c r="P1001" s="13"/>
+      <c r="Q1001" s="13"/>
+      <c r="R1001" s="13"/>
+      <c r="S1001" s="13"/>
+      <c r="T1001" s="13"/>
+      <c r="U1001" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
modified scrape_rbi to avoid getting blocked by RBI
</commit_message>
<xml_diff>
--- a/data/Links.xlsx
+++ b/data/Links.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="SEBI"/>
@@ -186,7 +186,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -205,6 +205,12 @@
       <sz val="11"/>
       <color rgb="FF1155cc"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
@@ -295,10 +301,10 @@
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -51836,13 +51842,13 @@
     <col min="2" max="2" style="5" width="48.86214285714286" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -51850,7 +51856,7 @@
         <v>22</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
@@ -51858,7 +51864,7 @@
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="3" t="s">
         <v>24</v>
       </c>
@@ -51866,7 +51872,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="3" t="s">
         <v>26</v>
       </c>
@@ -51874,7 +51880,7 @@
         <v>27</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="7"/>
       <c r="B6" s="7"/>
     </row>

</xml_diff>

<commit_message>
updated, rbi is removed from links excel
</commit_message>
<xml_diff>
--- a/data/Links.xlsx
+++ b/data/Links.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="SEBI"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="49">
   <si>
     <t>Companies Act</t>
   </si>
@@ -88,22 +88,7 @@
     <t>RBI</t>
   </si>
   <si>
-    <t>https://www.rbi.org.in/Scripts/NotificationUser.aspx</t>
-  </si>
-  <si>
-    <t>https://www.rbi.org.in/Scripts/BS_PressReleaseDisplay.aspx</t>
-  </si>
-  <si>
-    <t>Master Circular</t>
-  </si>
-  <si>
-    <t>https://www.rbi.org.in/Scripts/BS_ViewMasterCirculardetails.aspx</t>
-  </si>
-  <si>
-    <t>Master Directions</t>
-  </si>
-  <si>
-    <t>https://www.rbi.org.in/Scripts/BS_ViewMasterDirections.aspx</t>
+    <t/>
   </si>
   <si>
     <t>IFSCA - Gift</t>
@@ -172,6 +157,9 @@
     <t>https://www.sebi.gov.in/sebiweb/home/HomeAction.do?doListingLegal=yes&amp;sid=1&amp;ssid=3&amp;smid=0</t>
   </si>
   <si>
+    <t>Master Circular</t>
+  </si>
+  <si>
     <t>https://www.sebi.gov.in/sebiweb/home/HomeAction.do?doListing=yes&amp;sid=1&amp;ssid=6&amp;smid=0</t>
   </si>
   <si>
@@ -186,7 +174,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -205,12 +193,6 @@
       <sz val="11"/>
       <color rgb="FF1155cc"/>
       <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
@@ -272,7 +254,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -301,10 +283,16 @@
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -646,7 +634,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
@@ -678,7 +666,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
@@ -710,7 +698,7 @@
         <v>5</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -739,10 +727,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
       <c r="A4" s="3" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -774,7 +762,7 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
@@ -803,10 +791,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
       <c r="A6" s="3" t="s">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
@@ -835,10 +823,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
       <c r="A7" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -28708,7 +28696,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
@@ -28732,10 +28720,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
       <c r="A2" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
@@ -28759,10 +28747,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="3" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -28785,8 +28773,8 @@
       <c r="U3" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="10"/>
-      <c r="B4" s="11"/>
+      <c r="A4" s="12"/>
+      <c r="B4" s="13"/>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
@@ -51690,53 +51678,53 @@
       <c r="R999" s="7"/>
       <c r="S999" s="7"/>
       <c r="T999" s="7"/>
-      <c r="U999" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="1000" customHeight="1" ht="17.25" customFormat="1" s="12">
-      <c r="A1000" s="11"/>
+      <c r="U999" s="12"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="1000" customHeight="1" ht="17.25" customFormat="1" s="14">
+      <c r="A1000" s="13"/>
       <c r="B1000" s="8"/>
-      <c r="C1000" s="11"/>
-      <c r="D1000" s="11"/>
-      <c r="E1000" s="11"/>
-      <c r="F1000" s="11"/>
-      <c r="G1000" s="11"/>
-      <c r="H1000" s="11"/>
-      <c r="I1000" s="11"/>
-      <c r="J1000" s="11"/>
-      <c r="K1000" s="11"/>
-      <c r="L1000" s="11"/>
-      <c r="M1000" s="11"/>
-      <c r="N1000" s="11"/>
-      <c r="O1000" s="11"/>
-      <c r="P1000" s="11"/>
-      <c r="Q1000" s="11"/>
-      <c r="R1000" s="11"/>
-      <c r="S1000" s="11"/>
-      <c r="T1000" s="11"/>
-      <c r="U1000" s="11"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="1001" customHeight="1" ht="17.25" customFormat="1" s="12">
-      <c r="A1001" s="11"/>
+      <c r="C1000" s="13"/>
+      <c r="D1000" s="13"/>
+      <c r="E1000" s="13"/>
+      <c r="F1000" s="13"/>
+      <c r="G1000" s="13"/>
+      <c r="H1000" s="13"/>
+      <c r="I1000" s="13"/>
+      <c r="J1000" s="13"/>
+      <c r="K1000" s="13"/>
+      <c r="L1000" s="13"/>
+      <c r="M1000" s="13"/>
+      <c r="N1000" s="13"/>
+      <c r="O1000" s="13"/>
+      <c r="P1000" s="13"/>
+      <c r="Q1000" s="13"/>
+      <c r="R1000" s="13"/>
+      <c r="S1000" s="13"/>
+      <c r="T1000" s="13"/>
+      <c r="U1000" s="13"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="1001" customHeight="1" ht="17.25" customFormat="1" s="14">
+      <c r="A1001" s="13"/>
       <c r="B1001" s="8"/>
-      <c r="C1001" s="11"/>
-      <c r="D1001" s="11"/>
-      <c r="E1001" s="11"/>
-      <c r="F1001" s="11"/>
-      <c r="G1001" s="11"/>
-      <c r="H1001" s="11"/>
-      <c r="I1001" s="11"/>
-      <c r="J1001" s="11"/>
-      <c r="K1001" s="11"/>
-      <c r="L1001" s="11"/>
-      <c r="M1001" s="11"/>
-      <c r="N1001" s="11"/>
-      <c r="O1001" s="11"/>
-      <c r="P1001" s="11"/>
-      <c r="Q1001" s="11"/>
-      <c r="R1001" s="11"/>
-      <c r="S1001" s="11"/>
-      <c r="T1001" s="11"/>
-      <c r="U1001" s="11"/>
+      <c r="C1001" s="13"/>
+      <c r="D1001" s="13"/>
+      <c r="E1001" s="13"/>
+      <c r="F1001" s="13"/>
+      <c r="G1001" s="13"/>
+      <c r="H1001" s="13"/>
+      <c r="I1001" s="13"/>
+      <c r="J1001" s="13"/>
+      <c r="K1001" s="13"/>
+      <c r="L1001" s="13"/>
+      <c r="M1001" s="13"/>
+      <c r="N1001" s="13"/>
+      <c r="O1001" s="13"/>
+      <c r="P1001" s="13"/>
+      <c r="Q1001" s="13"/>
+      <c r="R1001" s="13"/>
+      <c r="S1001" s="13"/>
+      <c r="T1001" s="13"/>
+      <c r="U1001" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -51758,7 +51746,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
@@ -51766,7 +51754,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="30">
@@ -51774,7 +51762,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="30">
@@ -51782,7 +51770,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="30">
@@ -51790,7 +51778,7 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="30">
@@ -51798,23 +51786,23 @@
         <v>16</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="30">
       <c r="A7" s="3" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="30">
       <c r="A8" s="3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
@@ -51822,7 +51810,7 @@
         <v>12</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -51849,35 +51837,35 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4" t="s">
+      <c r="A2" s="10" t="s">
         <v>22</v>
       </c>
+      <c r="B2" s="11" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="3" t="s">
-        <v>5</v>
+      <c r="A3" s="10" t="s">
+        <v>22</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>23</v>
+      <c r="B3" s="11" t="s">
+        <v>22</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="3" t="s">
-        <v>24</v>
+      <c r="A4" s="10" t="s">
+        <v>22</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>25</v>
+      <c r="B4" s="11" t="s">
+        <v>22</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="3" t="s">
-        <v>26</v>
+      <c r="A5" s="10" t="s">
+        <v>22</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>27</v>
+      <c r="B5" s="11" t="s">
+        <v>22</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">

</xml_diff>

<commit_message>
fixed ICAI parsing agent
</commit_message>
<xml_diff>
--- a/data/Links.xlsx
+++ b/data/Links.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="3"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="SEBI"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="45">
   <si>
     <t>Companies Act</t>
   </si>
@@ -88,9 +88,6 @@
     <t>RBI</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>IFSCA - Gift</t>
   </si>
   <si>
@@ -127,16 +124,7 @@
     <t>Listed Companies</t>
   </si>
   <si>
-    <t>Circular-BSE</t>
-  </si>
-  <si>
-    <t>https://www.bseindia.com/corporates/CirularToListedComp.html</t>
-  </si>
-  <si>
-    <t>Circular-NSE</t>
-  </si>
-  <si>
-    <t>https://www.nseindia.com/companies-listing/circular-for-listed-companies-equity-market</t>
+    <t/>
   </si>
   <si>
     <t>SEBI</t>
@@ -634,7 +622,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
@@ -666,7 +654,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
@@ -698,7 +686,7 @@
         <v>5</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -727,10 +715,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
       <c r="A4" s="3" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -762,7 +750,7 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
@@ -791,10 +779,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
       <c r="A6" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
@@ -823,10 +811,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
       <c r="A7" s="3" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -28696,7 +28684,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
@@ -28719,11 +28707,11 @@
       <c r="U1" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
-      <c r="A2" s="3" t="s">
-        <v>35</v>
+      <c r="A2" s="10" t="s">
+        <v>34</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>36</v>
+      <c r="B2" s="11" t="s">
+        <v>34</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
@@ -28746,11 +28734,11 @@
       <c r="U2" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="3" t="s">
-        <v>37</v>
+      <c r="A3" s="10" t="s">
+        <v>34</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>38</v>
+      <c r="B3" s="11" t="s">
+        <v>34</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -51746,7 +51734,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
@@ -51754,7 +51742,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="30">
@@ -51762,7 +51750,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="30">
@@ -51770,7 +51758,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="30">
@@ -51778,7 +51766,7 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="30">
@@ -51786,23 +51774,23 @@
         <v>16</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="30">
+      <c r="A7" s="3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="30">
-      <c r="A7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="4" t="s">
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="30">
+      <c r="A8" s="3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="30">
-      <c r="A8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>31</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>32</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
@@ -51810,7 +51798,7 @@
         <v>12</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -51837,36 +51825,20 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>22</v>
-      </c>
+      <c r="A2" s="3"/>
+      <c r="B2" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>22</v>
-      </c>
+      <c r="A3" s="3"/>
+      <c r="B3" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>22</v>
-      </c>
+      <c r="A4" s="3"/>
+      <c r="B4" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>22</v>
-      </c>
+      <c r="A5" s="3"/>
+      <c r="B5" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="7"/>

</xml_diff>

<commit_message>
added ifsca informal guidance
</commit_message>
<xml_diff>
--- a/data/Links.xlsx
+++ b/data/Links.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="SEBI"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="45">
   <si>
     <t>Companies Act</t>
   </si>
@@ -121,10 +121,10 @@
     <t>https://ifsca.gov.in/Legal/Index/sKCVtbX6J9o=</t>
   </si>
   <si>
-    <t>Listed Companies</t>
+    <t/>
   </si>
   <si>
-    <t/>
+    <t>Listed Companies</t>
   </si>
   <si>
     <t>SEBI</t>
@@ -271,7 +271,7 @@
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
@@ -28684,7 +28684,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
@@ -28707,12 +28707,8 @@
       <c r="U1" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
-      <c r="A2" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>34</v>
-      </c>
+      <c r="A2" s="3"/>
+      <c r="B2" s="4"/>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
       <c r="E2" s="7"/>
@@ -28734,12 +28730,8 @@
       <c r="U2" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>34</v>
-      </c>
+      <c r="A3" s="3"/>
+      <c r="B3" s="4"/>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -51724,20 +51716,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="6" width="40.57642857142857" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -51745,7 +51737,7 @@
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="30">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
       <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
@@ -51753,7 +51745,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="30">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="31.5">
       <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
@@ -51761,7 +51753,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="30">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="31.5">
       <c r="A5" s="3" t="s">
         <v>10</v>
       </c>
@@ -51769,7 +51761,7 @@
         <v>26</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="30">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="31.5">
       <c r="A6" s="3" t="s">
         <v>16</v>
       </c>
@@ -51777,7 +51769,7 @@
         <v>27</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="30">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="31.5">
       <c r="A7" s="3" t="s">
         <v>28</v>
       </c>
@@ -51785,7 +51777,7 @@
         <v>29</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="30">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="31.5">
       <c r="A8" s="3" t="s">
         <v>30</v>
       </c>
@@ -51793,12 +51785,20 @@
         <v>31</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
       <c r="A9" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>32</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="31.5">
+      <c r="A10" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated to be ignore for rbi
</commit_message>
<xml_diff>
--- a/data/Links.xlsx
+++ b/data/Links.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="6"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="SEBI"/>
@@ -20,12 +20,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="41">
   <si>
     <t>Companies Act</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>IBBI - Litigation</t>
@@ -233,7 +230,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -241,10 +238,10 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -257,12 +254,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
@@ -613,7 +604,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
@@ -641,11 +632,11 @@
       <c r="Z1" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
-      <c r="A2" s="9" t="s">
-        <v>5</v>
+      <c r="A2" s="3" t="s">
+        <v>4</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>33</v>
+      <c r="B2" s="4" t="s">
+        <v>32</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
@@ -673,11 +664,11 @@
       <c r="Z2" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
-      <c r="A3" s="9" t="s">
-        <v>22</v>
+      <c r="A3" s="3" t="s">
+        <v>21</v>
       </c>
-      <c r="B3" s="10" t="s">
-        <v>34</v>
+      <c r="B3" s="4" t="s">
+        <v>33</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -705,11 +696,11 @@
       <c r="Z3" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="31.5">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>35</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>36</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -737,11 +728,11 @@
       <c r="Z4" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="31.5">
-      <c r="A5" s="9" t="s">
-        <v>7</v>
+      <c r="A5" s="3" t="s">
+        <v>6</v>
       </c>
-      <c r="B5" s="10" t="s">
-        <v>37</v>
+      <c r="B5" s="4" t="s">
+        <v>36</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
@@ -769,11 +760,11 @@
       <c r="Z5" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="31.5">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>38</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>39</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
@@ -801,11 +792,11 @@
       <c r="Z6" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="31.5">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>41</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -972,7 +963,7 @@
       <c r="Y12" s="7"/>
       <c r="Z12" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="7"/>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
@@ -1000,7 +991,7 @@
       <c r="Y13" s="7"/>
       <c r="Z13" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="7"/>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
@@ -1028,7 +1019,7 @@
       <c r="Y14" s="7"/>
       <c r="Z14" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="7"/>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
@@ -28675,7 +28666,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
@@ -28698,8 +28689,8 @@
       <c r="U1" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
-      <c r="A2" s="9"/>
-      <c r="B2" s="10"/>
+      <c r="A2" s="3"/>
+      <c r="B2" s="4"/>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
       <c r="E2" s="7"/>
@@ -28721,8 +28712,8 @@
       <c r="U2" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="9"/>
-      <c r="B3" s="10"/>
+      <c r="A3" s="3"/>
+      <c r="B3" s="4"/>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -28744,8 +28735,8 @@
       <c r="U3" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="12"/>
-      <c r="B4" s="13"/>
+      <c r="A4" s="10"/>
+      <c r="B4" s="11"/>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
@@ -51649,53 +51640,53 @@
       <c r="R999" s="7"/>
       <c r="S999" s="7"/>
       <c r="T999" s="7"/>
-      <c r="U999" s="12"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="1000" customHeight="1" ht="17.25" customFormat="1" s="14">
-      <c r="A1000" s="13"/>
+      <c r="U999" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="1000" customHeight="1" ht="17.25" customFormat="1" s="12">
+      <c r="A1000" s="11"/>
       <c r="B1000" s="8"/>
-      <c r="C1000" s="13"/>
-      <c r="D1000" s="13"/>
-      <c r="E1000" s="13"/>
-      <c r="F1000" s="13"/>
-      <c r="G1000" s="13"/>
-      <c r="H1000" s="13"/>
-      <c r="I1000" s="13"/>
-      <c r="J1000" s="13"/>
-      <c r="K1000" s="13"/>
-      <c r="L1000" s="13"/>
-      <c r="M1000" s="13"/>
-      <c r="N1000" s="13"/>
-      <c r="O1000" s="13"/>
-      <c r="P1000" s="13"/>
-      <c r="Q1000" s="13"/>
-      <c r="R1000" s="13"/>
-      <c r="S1000" s="13"/>
-      <c r="T1000" s="13"/>
-      <c r="U1000" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="1001" customHeight="1" ht="17.25" customFormat="1" s="14">
-      <c r="A1001" s="13"/>
+      <c r="C1000" s="11"/>
+      <c r="D1000" s="11"/>
+      <c r="E1000" s="11"/>
+      <c r="F1000" s="11"/>
+      <c r="G1000" s="11"/>
+      <c r="H1000" s="11"/>
+      <c r="I1000" s="11"/>
+      <c r="J1000" s="11"/>
+      <c r="K1000" s="11"/>
+      <c r="L1000" s="11"/>
+      <c r="M1000" s="11"/>
+      <c r="N1000" s="11"/>
+      <c r="O1000" s="11"/>
+      <c r="P1000" s="11"/>
+      <c r="Q1000" s="11"/>
+      <c r="R1000" s="11"/>
+      <c r="S1000" s="11"/>
+      <c r="T1000" s="11"/>
+      <c r="U1000" s="11"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="1001" customHeight="1" ht="17.25" customFormat="1" s="12">
+      <c r="A1001" s="11"/>
       <c r="B1001" s="8"/>
-      <c r="C1001" s="13"/>
-      <c r="D1001" s="13"/>
-      <c r="E1001" s="13"/>
-      <c r="F1001" s="13"/>
-      <c r="G1001" s="13"/>
-      <c r="H1001" s="13"/>
-      <c r="I1001" s="13"/>
-      <c r="J1001" s="13"/>
-      <c r="K1001" s="13"/>
-      <c r="L1001" s="13"/>
-      <c r="M1001" s="13"/>
-      <c r="N1001" s="13"/>
-      <c r="O1001" s="13"/>
-      <c r="P1001" s="13"/>
-      <c r="Q1001" s="13"/>
-      <c r="R1001" s="13"/>
-      <c r="S1001" s="13"/>
-      <c r="T1001" s="13"/>
-      <c r="U1001" s="13"/>
+      <c r="C1001" s="11"/>
+      <c r="D1001" s="11"/>
+      <c r="E1001" s="11"/>
+      <c r="F1001" s="11"/>
+      <c r="G1001" s="11"/>
+      <c r="H1001" s="11"/>
+      <c r="I1001" s="11"/>
+      <c r="J1001" s="11"/>
+      <c r="K1001" s="11"/>
+      <c r="L1001" s="11"/>
+      <c r="M1001" s="11"/>
+      <c r="N1001" s="11"/>
+      <c r="O1001" s="11"/>
+      <c r="P1001" s="11"/>
+      <c r="Q1001" s="11"/>
+      <c r="R1001" s="11"/>
+      <c r="S1001" s="11"/>
+      <c r="T1001" s="11"/>
+      <c r="U1001" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -51717,76 +51708,76 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
-      <c r="A2" s="9" t="s">
-        <v>3</v>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
+      <c r="A3" s="3" t="s">
+        <v>4</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B3" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
-      <c r="A3" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="10" t="s">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="31.5">
+      <c r="A4" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="31.5">
-      <c r="A4" s="9" t="s">
+      <c r="B4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="10" t="s">
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="31.5">
+      <c r="A5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="31.5">
-      <c r="A5" s="9" t="s">
-        <v>7</v>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="31.5">
+      <c r="A6" s="3" t="s">
+        <v>12</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B6" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="31.5">
-      <c r="A6" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="10" t="s">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="31.5">
+      <c r="A7" s="3" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="31.5">
-      <c r="A7" s="9" t="s">
+      <c r="B7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="10" t="s">
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="31.5">
+      <c r="A8" s="3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="31.5">
-      <c r="A8" s="9" t="s">
+      <c r="B8" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="10" t="s">
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
+      <c r="A9" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
-      <c r="A9" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>30</v>
-      </c>
-    </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="31.5">
       <c r="A10" s="7"/>
-      <c r="B10" s="10"/>
+      <c r="B10" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -51808,24 +51799,24 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="9"/>
-      <c r="B2" s="10"/>
+      <c r="A2" s="3"/>
+      <c r="B2" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="9"/>
-      <c r="B3" s="10"/>
+      <c r="A3" s="3"/>
+      <c r="B3" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="9"/>
-      <c r="B4" s="10"/>
+      <c r="A4" s="3"/>
+      <c r="B4" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="9"/>
-      <c r="B5" s="10"/>
+      <c r="A5" s="3"/>
+      <c r="B5" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="7"/>
@@ -51851,15 +51842,15 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
+      <c r="A2" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
-      <c r="A2" s="9" t="s">
+      <c r="B2" s="9" t="s">
         <v>16</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -51882,55 +51873,55 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
+      <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
-      <c r="A2" s="9" t="s">
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="10" t="s">
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
+      <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
-      <c r="A3" s="9" t="s">
+      <c r="B3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="10" t="s">
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
+      <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
-      <c r="A4" s="9" t="s">
+      <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="10" t="s">
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
+      <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
-      <c r="A5" s="9" t="s">
+      <c r="B5" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="11" t="s">
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
+      <c r="A6" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
-      <c r="A6" s="9" t="s">
+      <c r="B6" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="11" t="s">
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
+      <c r="A7" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
-      <c r="A7" s="9" t="s">
+      <c r="B7" s="4" t="s">
         <v>13</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -51957,28 +51948,16 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A2" s="3"/>
+      <c r="B2" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
-      <c r="A3" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A3" s="3"/>
+      <c r="B3" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="44.25">
-      <c r="A4" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A4" s="3"/>
+      <c r="B4" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
made chrome version more dynamic in mca and listed companies
</commit_message>
<xml_diff>
--- a/data/Links.xlsx
+++ b/data/Links.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="SEBI"/>
@@ -51870,13 +51870,13 @@
     <col min="2" max="2" style="5" width="41.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -51884,7 +51884,7 @@
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -51892,7 +51892,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="31.5">
       <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
@@ -51900,7 +51900,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
@@ -51908,7 +51908,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="3" t="s">
         <v>10</v>
       </c>
@@ -51916,7 +51916,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="31.5">
       <c r="A7" s="3" t="s">
         <v>12</v>
       </c>

</xml_diff>

<commit_message>
added links of mca,rbi,ifsca IG back to main pipeline
</commit_message>
<xml_diff>
--- a/data/Links.xlsx
+++ b/data/Links.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="SEBI"/>
@@ -20,21 +20,33 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="50">
   <si>
     <t>Companies Act</t>
+  </si>
+  <si>
+    <t>Notifications</t>
+  </si>
+  <si>
+    <t>https://www.mca.gov.in/content/mca/global/en/acts-rules/ebooks/notifications.html</t>
+  </si>
+  <si>
+    <t>Circulars</t>
+  </si>
+  <si>
+    <t>https://www.mca.gov.in/content/mca/global/en/acts-rules/ebooks/circulars.html</t>
+  </si>
+  <si>
+    <t>Press Release</t>
+  </si>
+  <si>
+    <t>https://www.mca.gov.in/content/mca/global/en/notifications-tender/news-updates/press-release.html</t>
   </si>
   <si>
     <t>IBBI - Litigation</t>
   </si>
   <si>
-    <t>Notifications</t>
-  </si>
-  <si>
     <t>https://ibbi.gov.in//en/legal-framework/notifications</t>
-  </si>
-  <si>
-    <t>Circulars</t>
   </si>
   <si>
     <t>https://ibbi.gov.in//en/legal-framework/circulars</t>
@@ -76,6 +88,24 @@
     <t>RBI</t>
   </si>
   <si>
+    <t>https://www.rbi.org.in/Scripts/NotificationUser.aspx</t>
+  </si>
+  <si>
+    <t>https://www.rbi.org.in/Scripts/BS_PressReleaseDisplay.aspx</t>
+  </si>
+  <si>
+    <t>Master Circular</t>
+  </si>
+  <si>
+    <t>https://www.rbi.org.in/Scripts/BS_ViewMasterCirculardetails.aspx</t>
+  </si>
+  <si>
+    <t>Master Directions</t>
+  </si>
+  <si>
+    <t>https://www.rbi.org.in/Scripts/BS_ViewMasterDirections.aspx</t>
+  </si>
+  <si>
     <t>IFSCA - Gift</t>
   </si>
   <si>
@@ -83,9 +113,6 @@
   </si>
   <si>
     <t>https://ifsca.gov.in/Legal/Index/wF6kttc1JR8=</t>
-  </si>
-  <si>
-    <t>Press Release</t>
   </si>
   <si>
     <t>https://ifsca.gov.in/PressRelease/Index/MEdJSLhva0M=</t>
@@ -112,6 +139,12 @@
     <t>https://ifsca.gov.in/Legal/Index/sKCVtbX6J9o=</t>
   </si>
   <si>
+    <t>Informal Guidance</t>
+  </si>
+  <si>
+    <t>https://ifsca.gov.in/InformalGuidance/Index</t>
+  </si>
+  <si>
     <t>Listed Companies</t>
   </si>
   <si>
@@ -133,13 +166,7 @@
     <t>https://www.sebi.gov.in/sebiweb/home/HomeAction.do?doListingLegal=yes&amp;sid=1&amp;ssid=3&amp;smid=0</t>
   </si>
   <si>
-    <t>Master Circular</t>
-  </si>
-  <si>
     <t>https://www.sebi.gov.in/sebiweb/home/HomeAction.do?doListing=yes&amp;sid=1&amp;ssid=6&amp;smid=0</t>
-  </si>
-  <si>
-    <t>Informal Guidance</t>
   </si>
   <si>
     <t>https://www.sebi.gov.in/sebiweb/home/HomeAction.do?doListing=yes&amp;sid=2&amp;ssid=10&amp;smid=0</t>
@@ -604,7 +631,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
@@ -633,10 +660,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
       <c r="A2" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
@@ -665,10 +692,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
       <c r="A3" s="3" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -697,10 +724,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="31.5">
       <c r="A4" s="3" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -729,10 +756,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="31.5">
       <c r="A5" s="3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
@@ -761,10 +788,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="31.5">
       <c r="A6" s="3" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
@@ -796,7 +823,7 @@
         <v>39</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -28666,7 +28693,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
@@ -51708,76 +51735,80 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
       <c r="A2" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
       <c r="A3" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="31.5">
       <c r="A4" s="3" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="31.5">
       <c r="A5" s="3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="31.5">
       <c r="A6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="31.5">
+      <c r="A7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="31.5">
+      <c r="A8" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
+      <c r="A9" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>24</v>
+      <c r="B9" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="31.5">
-      <c r="A7" s="3" t="s">
-        <v>25</v>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="31.5">
+      <c r="A10" s="7" t="s">
+        <v>39</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>26</v>
+      <c r="B10" s="4" t="s">
+        <v>40</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="31.5">
-      <c r="A8" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
-      <c r="A9" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="31.5">
-      <c r="A10" s="7"/>
-      <c r="B10" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -51799,24 +51830,40 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="3"/>
-      <c r="B2" s="4"/>
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
+      <c r="A3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4"/>
+      <c r="A4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4"/>
+      <c r="A5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="7"/>
@@ -51842,15 +51889,15 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
       <c r="A2" s="3" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -51873,55 +51920,55 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
-      <c r="A2" s="3" t="s">
-        <v>2</v>
+      <c r="B2" s="4" t="s">
+        <v>8</v>
       </c>
-      <c r="B2" s="4" t="s">
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
+      <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
-      <c r="A3" s="3" t="s">
-        <v>4</v>
-      </c>
       <c r="B3" s="4" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="31.5">
       <c r="A4" s="3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="3" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="3" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="31.5">
       <c r="A7" s="3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -51948,16 +51995,28 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
-      <c r="A2" s="3"/>
-      <c r="B2" s="4"/>
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
+      <c r="A3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="44.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4"/>
+      <c r="A4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>